<commit_message>
Preserve specific issue highlights on duplicate rows
</commit_message>
<xml_diff>
--- a/reviewed_sample_jobs.xlsx
+++ b/reviewed_sample_jobs.xlsx
@@ -74,8 +74,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -537,7 +537,7 @@
           <t>charlie@example.com</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>temporary</t>
         </is>
@@ -562,12 +562,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Highlight</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
@@ -582,7 +582,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Invalid value</t>

</xml_diff>

<commit_message>
Polish annotated workbook output
</commit_message>
<xml_diff>
--- a/reviewed_sample_jobs.xlsx
+++ b/reviewed_sample_jobs.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$D$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -28,9 +30,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -39,22 +42,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
+        <fgColor rgb="FF44546A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF9999"/>
+        <fgColor rgb="FFF7F7F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD699"/>
+        <fgColor rgb="FFFCE5CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,13 +83,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -151,6 +165,31 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Data Quality Toolkit</author>
+  </authors>
+  <commentList>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>Missing required value.</t>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="0" shapeId="0">
+      <text>
+        <t>Duplicate record detected.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Invalid value: temporary</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -444,44 +483,50 @@
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>employment_type</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>alice@example.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>full-time</t>
         </is>
@@ -508,43 +553,45 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>103</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Charlie</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>contract</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>103</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Charlie</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>charlie@example.com</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>temporary</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -558,23 +605,23 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Highlight</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr"/>
+      <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Missing required value</t>
@@ -582,7 +629,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
+      <c r="A3" s="5" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Invalid value</t>
@@ -590,7 +637,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Duplicate row</t>
@@ -598,7 +645,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
+      <c r="A5" s="6" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Unexpected column</t>

</xml_diff>